<commit_message>
finish template for creek by blood minor
</commit_message>
<xml_diff>
--- a/DawesRollsViewer/Dawes Rolls One Document/Creek/Creek Minor By Blood.xlsx
+++ b/DawesRollsViewer/Dawes Rolls One Document/Creek/Creek Minor By Blood.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="25">
   <si>
     <t>ID</t>
   </si>
@@ -83,6 +83,12 @@
   </si>
   <si>
     <t>Image Binary</t>
+  </si>
+  <si>
+    <t>Stricken from roll</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -8141,8 +8147,35 @@
         <f t="shared" si="18"/>
         <v>573</v>
       </c>
+      <c r="D385" t="s">
+        <v>23</v>
+      </c>
+      <c r="E385" t="s">
+        <v>24</v>
+      </c>
+      <c r="F385" t="s">
+        <v>24</v>
+      </c>
+      <c r="G385" t="s">
+        <v>24</v>
+      </c>
+      <c r="H385">
+        <v>-1</v>
+      </c>
+      <c r="I385" t="s">
+        <v>24</v>
+      </c>
+      <c r="J385" t="s">
+        <v>24</v>
+      </c>
+      <c r="K385" t="s">
+        <v>24</v>
+      </c>
       <c r="L385" t="s">
-        <v>16</v>
+        <v>24</v>
+      </c>
+      <c r="M385" t="s">
+        <v>24</v>
       </c>
       <c r="N385" t="str">
         <f t="shared" si="19"/>
@@ -8161,8 +8194,35 @@
         <f t="shared" si="18"/>
         <v>573</v>
       </c>
+      <c r="D386" t="s">
+        <v>23</v>
+      </c>
+      <c r="E386" t="s">
+        <v>24</v>
+      </c>
+      <c r="F386" t="s">
+        <v>24</v>
+      </c>
+      <c r="G386" t="s">
+        <v>24</v>
+      </c>
+      <c r="H386">
+        <v>0</v>
+      </c>
+      <c r="I386" t="s">
+        <v>24</v>
+      </c>
+      <c r="J386" t="s">
+        <v>24</v>
+      </c>
+      <c r="K386" t="s">
+        <v>24</v>
+      </c>
       <c r="L386" t="s">
-        <v>16</v>
+        <v>24</v>
+      </c>
+      <c r="M386" t="s">
+        <v>24</v>
       </c>
       <c r="N386" t="str">
         <f t="shared" si="19"/>
@@ -8181,8 +8241,35 @@
         <f t="shared" si="18"/>
         <v>573</v>
       </c>
+      <c r="D387" t="s">
+        <v>23</v>
+      </c>
+      <c r="E387" t="s">
+        <v>24</v>
+      </c>
+      <c r="F387" t="s">
+        <v>24</v>
+      </c>
+      <c r="G387" t="s">
+        <v>24</v>
+      </c>
+      <c r="H387">
+        <v>1</v>
+      </c>
+      <c r="I387" t="s">
+        <v>24</v>
+      </c>
+      <c r="J387" t="s">
+        <v>24</v>
+      </c>
+      <c r="K387" t="s">
+        <v>24</v>
+      </c>
       <c r="L387" t="s">
-        <v>16</v>
+        <v>24</v>
+      </c>
+      <c r="M387" t="s">
+        <v>24</v>
       </c>
       <c r="N387" t="str">
         <f t="shared" si="19"/>

</xml_diff>